<commit_message>
repairer added and insurer is updated
</commit_message>
<xml_diff>
--- a/Test Data/ICGMS Test Data.xlsx
+++ b/Test Data/ICGMS Test Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Parth Grover\Desktop\DTU\Sharajman Work\automation-icgms\Test Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C144EF5A-463E-418C-8BEB-D9B5730049F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDC75072-C385-426C-B4B0-A7E5AF809CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="719" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="719" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MotorClaim_Insurer" sheetId="4" r:id="rId1"/>
@@ -950,7 +950,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>0</v>

</xml_diff>

<commit_message>
new pytest files added
</commit_message>
<xml_diff>
--- a/Test Data/ICGMS Test Data.xlsx
+++ b/Test Data/ICGMS Test Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Parth Grover\Desktop\DTU\Sharajman Work\automation-icgms\Test Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDC75072-C385-426C-B4B0-A7E5AF809CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC12114-F3A9-4248-9FD4-1565ECFCD602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="719" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="719" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MotorClaim_Insurer" sheetId="4" r:id="rId1"/>
@@ -867,7 +867,7 @@
     </row>
     <row r="2" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>0</v>
@@ -950,7 +950,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>0</v>

</xml_diff>

<commit_message>
Test data fields updated
</commit_message>
<xml_diff>
--- a/Test Data/ICGMS Test Data.xlsx
+++ b/Test Data/ICGMS Test Data.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Parth Grover\Desktop\DTU\Sharajman Work\automation-icgms\Test Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC12114-F3A9-4248-9FD4-1565ECFCD602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8446274F-DE9B-4501-B61C-070FB04EC1DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="719" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="719" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MotorClaim_Insurer" sheetId="4" r:id="rId1"/>
     <sheet name="PreInspection_Type" sheetId="7" r:id="rId2"/>
     <sheet name="SuperAdmin" sheetId="1" r:id="rId3"/>
     <sheet name="Customer" sheetId="2" r:id="rId4"/>
-    <sheet name="Repairer" sheetId="3" r:id="rId5"/>
-    <sheet name="Surveyor" sheetId="6" r:id="rId6"/>
+    <sheet name="Surveyor" sheetId="6" r:id="rId5"/>
+    <sheet name="Repairer" sheetId="3" r:id="rId6"/>
     <sheet name="Insurer_Log" sheetId="5" r:id="rId7"/>
   </sheets>
   <definedNames>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="65">
   <si>
     <t>Admin123</t>
   </si>
@@ -225,14 +225,17 @@
     <t>hepaybin@via.tokyo.jp</t>
   </si>
   <si>
-    <t>H@Z3J8QA</t>
+    <t>x@F2alq3</t>
+  </si>
+  <si>
+    <t>royalsundram@insurer.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -253,6 +256,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -371,8 +380,8 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -867,7 +876,7 @@
     </row>
     <row r="2" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>0</v>
@@ -949,8 +958,8 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
-        <v>60</v>
+      <c r="A2" s="12" t="s">
+        <v>39</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>0</v>
@@ -1097,6 +1106,58 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E41ABD4A-1C7D-4BEA-8306-D714B0819D20}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="46.109375" customWidth="1"/>
+    <col min="2" max="2" width="26.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" s="1"/>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2" xr:uid="{6BEFE3BA-BBEE-4D8D-8D2B-E98E86D98E53}">
+      <formula1>$A$3:$A$4</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{2552C37B-A202-4580-8249-8E7209909168}">
+      <formula1>$B$3:$B$4</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{450F6CC7-1659-4DFD-83EC-CFC4B11FFDB1}">
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1155,58 +1216,6 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2" xr:uid="{BC8FA23B-076C-4C85-AA74-2D83E1AD4459}">
       <formula1>$A$3:$A$6</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E41ABD4A-1C7D-4BEA-8306-D714B0819D20}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="46.109375" customWidth="1"/>
-    <col min="2" max="2" width="26.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B4" s="1"/>
-    </row>
-  </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2" xr:uid="{6BEFE3BA-BBEE-4D8D-8D2B-E98E86D98E53}">
-      <formula1>$A$3:$A$4</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{2552C37B-A202-4580-8249-8E7209909168}">
-      <formula1>$B$3:$B$4</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1247,7 +1256,9 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="1"/>
+      <c r="A4" s="1" t="s">
+        <v>64</v>
+      </c>
       <c r="B4" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert "Test data fields updated"
This reverts commit 1ae930532a83bcaca15268f8915b0c4de029fb71.
</commit_message>
<xml_diff>
--- a/Test Data/ICGMS Test Data.xlsx
+++ b/Test Data/ICGMS Test Data.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Parth Grover\Desktop\DTU\Sharajman Work\automation-icgms\Test Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8446274F-DE9B-4501-B61C-070FB04EC1DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC12114-F3A9-4248-9FD4-1565ECFCD602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="719" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="719" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MotorClaim_Insurer" sheetId="4" r:id="rId1"/>
     <sheet name="PreInspection_Type" sheetId="7" r:id="rId2"/>
     <sheet name="SuperAdmin" sheetId="1" r:id="rId3"/>
     <sheet name="Customer" sheetId="2" r:id="rId4"/>
-    <sheet name="Surveyor" sheetId="6" r:id="rId5"/>
-    <sheet name="Repairer" sheetId="3" r:id="rId6"/>
+    <sheet name="Repairer" sheetId="3" r:id="rId5"/>
+    <sheet name="Surveyor" sheetId="6" r:id="rId6"/>
     <sheet name="Insurer_Log" sheetId="5" r:id="rId7"/>
   </sheets>
   <definedNames>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="64">
   <si>
     <t>Admin123</t>
   </si>
@@ -225,17 +225,14 @@
     <t>hepaybin@via.tokyo.jp</t>
   </si>
   <si>
-    <t>x@F2alq3</t>
-  </si>
-  <si>
-    <t>royalsundram@insurer.com</t>
+    <t>H@Z3J8QA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -256,12 +253,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF333333"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -380,8 +371,8 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -876,7 +867,7 @@
     </row>
     <row r="2" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>0</v>
@@ -958,8 +949,8 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
-        <v>39</v>
+      <c r="A2" s="4" t="s">
+        <v>60</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>0</v>
@@ -1106,6 +1097,71 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{450F6CC7-1659-4DFD-83EC-CFC4B11FFDB1}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="46.109375" customWidth="1"/>
+    <col min="2" max="2" width="26.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B4" s="1"/>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="1"/>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="1"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{2D08C1CE-8B77-4399-AE61-B37DE842DDBE}">
+      <formula1>$B$3:$B$6</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2" xr:uid="{BC8FA23B-076C-4C85-AA74-2D83E1AD4459}">
+      <formula1>$A$3:$A$6</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E41ABD4A-1C7D-4BEA-8306-D714B0819D20}">
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1151,71 +1207,6 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{2552C37B-A202-4580-8249-8E7209909168}">
       <formula1>$B$3:$B$4</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{450F6CC7-1659-4DFD-83EC-CFC4B11FFDB1}">
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="46.109375" customWidth="1"/>
-    <col min="2" max="2" width="26.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B4" s="1"/>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>56</v>
-      </c>
-      <c r="B5" s="1"/>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" s="1"/>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{2D08C1CE-8B77-4399-AE61-B37DE842DDBE}">
-      <formula1>$B$3:$B$6</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2" xr:uid="{BC8FA23B-076C-4C85-AA74-2D83E1AD4459}">
-      <formula1>$A$3:$A$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1256,9 +1247,7 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>64</v>
-      </c>
+      <c r="A4" s="1"/>
       <c r="B4" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
base initiate and data updated
</commit_message>
<xml_diff>
--- a/Test Data/ICGMS Test Data.xlsx
+++ b/Test Data/ICGMS Test Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Parth Grover\Desktop\DTU\Sharajman Work\automation-icgms\Test Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC12114-F3A9-4248-9FD4-1565ECFCD602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7741B4D-6E57-4F9D-ABD8-471473DD88CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="719" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="719" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MotorClaim_Insurer" sheetId="4" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="65">
   <si>
     <t>Admin123</t>
   </si>
@@ -226,6 +226,9 @@
   </si>
   <si>
     <t>H@Z3J8QA</t>
+  </si>
+  <si>
+    <t>royalsundram@insurer.com</t>
   </si>
 </sst>
 </file>
@@ -346,7 +349,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -373,6 +376,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -867,7 +871,7 @@
     </row>
     <row r="2" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>0</v>
@@ -950,7 +954,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>60</v>
+        <v>13</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>0</v>
@@ -1247,7 +1251,9 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="1"/>
+      <c r="A4" s="14" t="s">
+        <v>64</v>
+      </c>
       <c r="B4" s="1"/>
     </row>
   </sheetData>

</xml_diff>